<commit_message>
auto: skill更新を自動保存 (2026-08-07 10:05)
</commit_message>
<xml_diff>
--- a/examples/hearing-sheet-improved.xlsx
+++ b/examples/hearing-sheet-improved.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E43"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -575,7 +575,7 @@
           <t>会社名・屋号</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr"/>
+      <c r="D2" s="5" t="n"/>
       <c r="E2" s="4" t="inlineStr">
         <is>
           <t>正式名称でご記入ください</t>
@@ -586,13 +586,13 @@
       <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="n"/>
       <c r="C3" s="4" t="inlineStr">
         <is>
           <t>ご担当者名・部署・連絡先</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr"/>
+      <c r="D3" s="5" t="n"/>
       <c r="E3" s="4" t="inlineStr">
         <is>
           <t>主な窓口になる方</t>
@@ -603,13 +603,13 @@
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="n"/>
       <c r="C4" s="4" t="inlineStr">
         <is>
           <t>今回つくるもの</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr"/>
+      <c r="D4" s="5" t="n"/>
       <c r="E4" s="4" t="inlineStr">
         <is>
           <t>新規サイト / リニューアル / LP(1枚もの) / その他</t>
@@ -620,13 +620,13 @@
       <c r="A5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="n"/>
       <c r="C5" s="4" t="inlineStr">
         <is>
           <t>業種・主な商品やサービス</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr"/>
+      <c r="D5" s="5" t="n"/>
       <c r="E5" s="4" t="inlineStr">
         <is>
           <t>一言で「何屋さんか」が伝わるように</t>
@@ -637,13 +637,13 @@
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="n"/>
       <c r="C6" s="4" t="inlineStr">
         <is>
           <t>主なお客様は企業か個人か</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr"/>
+      <c r="D6" s="5" t="n"/>
       <c r="E6" s="4" t="inlineStr">
         <is>
           <t>BtoB(企業) / BtoC(個人) / 両方</t>
@@ -654,13 +654,13 @@
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="n"/>
       <c r="C7" s="4" t="inlineStr">
         <is>
           <t>公開したい時期</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr"/>
+      <c r="D7" s="5" t="n"/>
       <c r="E7" s="4" t="inlineStr">
         <is>
           <t>「〇月頃」「特になし」など</t>
@@ -671,13 +671,13 @@
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="n"/>
       <c r="C8" s="4" t="inlineStr">
         <is>
           <t>ご予算の目安</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr"/>
+      <c r="D8" s="5" t="n"/>
       <c r="E8" s="4" t="inlineStr">
         <is>
           <t>制作費の上限イメージ。未定なら「未定」で可</t>
@@ -688,13 +688,13 @@
       <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="n"/>
       <c r="C9" s="4" t="inlineStr">
         <is>
           <t>公開後の更新体制</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr"/>
+      <c r="D9" s="5" t="n"/>
       <c r="E9" s="4" t="inlineStr">
         <is>
           <t>社内で更新する人がいるか / 制作側に任せたいか</t>
@@ -715,7 +715,7 @@
           <t>このサイトで一番達成したいこと</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="n"/>
       <c r="E10" s="4" t="inlineStr">
         <is>
           <t>例: 問い合わせを増やす / 信頼を高める / 採用を強化</t>
@@ -726,13 +726,13 @@
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="n"/>
       <c r="C11" s="4" t="inlineStr">
         <is>
           <t>成果をどう測りたいか</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="n"/>
       <c r="E11" s="4" t="inlineStr">
         <is>
           <t>例: 月の問い合わせ件数 / 資料請求数 / 売上</t>
@@ -743,13 +743,13 @@
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="n"/>
       <c r="C12" s="4" t="inlineStr">
         <is>
           <t>今の集客・問い合わせの状況</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="n"/>
       <c r="E12" s="4" t="inlineStr">
         <is>
           <t>例: 月に何件くらい / 主にどこから来るか</t>
@@ -760,13 +760,13 @@
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="n"/>
       <c r="C13" s="4" t="inlineStr">
         <is>
           <t>(リニューアル)今のサイトの不満・課題</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr"/>
+      <c r="D13" s="5" t="n"/>
       <c r="E13" s="4" t="inlineStr">
         <is>
           <t>見た目 / 使いにくさ / 成果が出ない など</t>
@@ -777,20 +777,16 @@
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>C.ブランドの核</t>
-        </is>
-      </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>お客様に最終的に「どう思われたいか」</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr"/>
+      <c r="B14" s="4" t="n"/>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>(リニューアル)今のサイトの数字</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n"/>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>一言で。例: 信頼できる / 頼れる / 一歩先を行く ★デザインの拠り所になります</t>
+          <t>分かる範囲で結構です。月にどれくらい見られているか / 検索でどんな言葉から来ているか / すぐ帰ってしまう人の割合 / よく見られているページ。アクセス解析(Googleアナリティクス等)の画面共有でもOK ★課題を「感覚」でなく数字で示せます</t>
         </is>
       </c>
     </row>
@@ -798,16 +794,20 @@
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="4" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>C.ブランドの核</t>
+        </is>
+      </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>大事にしている価値・創業の想い</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr"/>
+          <t>お客様に今「どう思われている」と感じるか</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n"/>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>なぜこの仕事をしているか。短くてOK ★コンセプトの根拠に使います</t>
+          <t>現状の印象を率直に。例: 古そう / 何屋さんか分からない / お高そう ★理想とのギャップが提案の出発点になります</t>
         </is>
       </c>
     </row>
@@ -815,16 +815,16 @@
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="n"/>
       <c r="C16" s="6" t="inlineStr">
         <is>
-          <t>ブランドを「人」に例えると？</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr"/>
+          <t>お客様に最終的に「どう思われたいか」</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n"/>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>例: 寡黙な職人 / 頼れる相棒 / 優しい先生 / 挑戦者 から近いものを</t>
+          <t>一言で。例: 信頼できる / 頼れる / 一歩先を行く ★デザインの拠り所になります</t>
         </is>
       </c>
     </row>
@@ -832,20 +832,16 @@
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="3" t="inlineStr">
-        <is>
-          <t>D.お客様(ターゲット)</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
-        <is>
-          <t>主なお客様はどんな方か</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr"/>
+      <c r="B17" s="4" t="n"/>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>大事にしている価値・創業の想い</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n"/>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>業種・規模・年齢・地域など分かる範囲で</t>
+          <t>なぜこの仕事をしているか。短くてOK ★コンセプトの根拠に使います</t>
         </is>
       </c>
     </row>
@@ -853,16 +849,16 @@
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="4" t="inlineStr"/>
-      <c r="C18" s="4" t="inlineStr">
-        <is>
-          <t>(BtoB)社内で誰が関わるか</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr"/>
+      <c r="B18" s="4" t="n"/>
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>ブランドを「人」に例えると？</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n"/>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>決める人 / 選ぶ担当者 / 実際に使う人</t>
+          <t>例: 寡黙な職人 / 頼れる相棒 / 優しい先生 / 挑戦者 から近いものを</t>
         </is>
       </c>
     </row>
@@ -870,16 +866,20 @@
       <c r="A19" s="2" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="4" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>D.お客様(ターゲット)</t>
+        </is>
+      </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>お客様の悩み・困りごと</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr"/>
+          <t>主なお客様はどんな方か</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n"/>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>それをサイトで解決できると刺さります</t>
+          <t>業種・規模・年齢・地域など分かる範囲で</t>
         </is>
       </c>
     </row>
@@ -887,16 +887,16 @@
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="4" t="inlineStr"/>
+      <c r="B20" s="4" t="n"/>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>選ぶときにお客様が不安に思うこと</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr"/>
+          <t>(BtoB)社内で誰が関わるか</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="n"/>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>例: 品質 / 実績 / 価格が分からない など</t>
+          <t>決める人 / 選ぶ担当者 / 実際に使う人</t>
         </is>
       </c>
     </row>
@@ -904,16 +904,16 @@
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="4" t="inlineStr"/>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>(BtoC)お客様自身が「こうありたい」姿</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr"/>
+      <c r="B21" s="4" t="n"/>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>お客様の悩み・困りごと</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="n"/>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>お客様が憧れる・なりたいイメージ ★その姿にデザインを寄せます</t>
+          <t>それをサイトで解決できると刺さります</t>
         </is>
       </c>
     </row>
@@ -921,20 +921,16 @@
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>E.強み・差別化</t>
-        </is>
-      </c>
+      <c r="B22" s="4" t="n"/>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>他社と比べた強み・選ばれる理由</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr"/>
+          <t>選ぶときにお客様が不安に思うこと</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="n"/>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>3つほど挙げてください</t>
+          <t>例: 品質 / 実績 / 価格が分からない など</t>
         </is>
       </c>
     </row>
@@ -942,16 +938,16 @@
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
-      <c r="B23" s="4" t="inlineStr"/>
-      <c r="C23" s="4" t="inlineStr">
-        <is>
-          <t>出せる実績・事例</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr"/>
+      <c r="B23" s="4" t="n"/>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>(BtoC)お客様自身が「こうありたい」姿</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="n"/>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>件数 / 社名を出してよいか / 写真の有無</t>
+          <t>お客様が憧れる・なりたいイメージ ★その姿にデザインを寄せます</t>
         </is>
       </c>
     </row>
@@ -959,16 +955,20 @@
       <c r="A24" s="2" t="n">
         <v>23</v>
       </c>
-      <c r="B24" s="4" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>E.強み・差別化</t>
+        </is>
+      </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>料金をサイトに載せられるか</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr"/>
+          <t>他社と比べた強み・選ばれる理由</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="n"/>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>載せる / 一部のみ / 載せない</t>
+          <t>3つほど挙げてください</t>
         </is>
       </c>
     </row>
@@ -976,20 +976,16 @@
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>F.競合・参考サイト</t>
-        </is>
-      </c>
+      <c r="B25" s="4" t="n"/>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>競合だと思う会社・サイト</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr"/>
+          <t>出せる実績・事例</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="n"/>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>URLがあれば(複数可)</t>
+          <t>件数 / 社名を出してよいか / 写真の有無</t>
         </is>
       </c>
     </row>
@@ -997,16 +993,16 @@
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
-      <c r="B26" s="4" t="inlineStr"/>
+      <c r="B26" s="4" t="n"/>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>参考にしたい・好きなサイト</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr"/>
+          <t>料金をサイトに載せられるか</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="n"/>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>URLと「どこが良いか」も一言</t>
+          <t>載せる / 一部のみ / 載せない</t>
         </is>
       </c>
     </row>
@@ -1014,16 +1010,20 @@
       <c r="A27" s="2" t="n">
         <v>26</v>
       </c>
-      <c r="B27" s="4" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>F.競合・参考サイト</t>
+        </is>
+      </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>こうはしたくない例</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr"/>
+          <t>競合だと思う会社・サイト</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="n"/>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>避けたい雰囲気 / 他社のNG例</t>
+          <t>URLがあれば(複数可)</t>
         </is>
       </c>
     </row>
@@ -1031,16 +1031,16 @@
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
-      <c r="B28" s="4" t="inlineStr"/>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>競合と「見た目で」どう差をつけたいか</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr"/>
+      <c r="B28" s="4" t="n"/>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>参考にしたい・好きなサイト</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="n"/>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>例: 競合より落ち着かせたい / 親しみを出したい ★同質化を避ける指針に</t>
+          <t>URLと「どこが良いか」も一言</t>
         </is>
       </c>
     </row>
@@ -1048,20 +1048,16 @@
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
-      <c r="B29" s="3" t="inlineStr">
-        <is>
-          <t>G.コンテンツ・機能</t>
-        </is>
-      </c>
+      <c r="B29" s="4" t="n"/>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>すでにある素材</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr"/>
+          <t>こうはしたくない例</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="n"/>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>ロゴ / 写真 / 文章 / パンフレット など</t>
+          <t>避けたい雰囲気 / 他社のNG例</t>
         </is>
       </c>
     </row>
@@ -1069,16 +1065,16 @@
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
-      <c r="B30" s="4" t="inlineStr"/>
-      <c r="C30" s="4" t="inlineStr">
-        <is>
-          <t>サイトに載せたいページ・内容</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr"/>
+      <c r="B30" s="4" t="n"/>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>競合と「見た目で」どう差をつけたいか</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="n"/>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>思いつくものを自由に</t>
+          <t>例: 競合より落ち着かせたい / 親しみを出したい ★同質化を避ける指針に</t>
         </is>
       </c>
     </row>
@@ -1086,16 +1082,20 @@
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
-      <c r="B31" s="4" t="inlineStr"/>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>G.素材・コンテンツ・機能</t>
+        </is>
+      </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>必要な機能</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr"/>
+          <t>【素材】ロゴのデータはありますか</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="n"/>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>問い合わせフォーム / 予約 / ブログ / ネット販売 など</t>
+          <t>当てはまるものを選んでください: イラストレーター形式(.ai)がある / それ以外の画像だけ(jpg・png等) / データが見当たらない ★.aiが無いと作り直しが必要になることがあります</t>
         </is>
       </c>
     </row>
@@ -1103,16 +1103,16 @@
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
-      <c r="B32" s="4" t="inlineStr"/>
+      <c r="B32" s="4" t="n"/>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>必須の掲載事項</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr"/>
+          <t>【素材】写真はありますか</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="n"/>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>会社情報 / 資格・許認可 / 法定表記 など</t>
+          <t>当てはまるものを選んでください: 支給できる写真がある(だいたい何点か) / これから撮影する / 用意がない(素材写真の購入を検討) ★使用できる期限があればあわせて</t>
         </is>
       </c>
     </row>
@@ -1120,20 +1120,16 @@
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
-      <c r="B33" s="3" t="inlineStr">
-        <is>
-          <t>H.デザインの希望</t>
-        </is>
-      </c>
+      <c r="B33" s="4" t="n"/>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>サイトの雰囲気・トーン</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr"/>
+          <t>【素材】パンフレット・チラシ・名刺などはありますか</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="n"/>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>別シート「トーン診断」もあわせてご記入ください</t>
+          <t>当てはまるものを選んでください: 印刷物だけある / データもある / 特にない ★見た目のトーンを合わせる手がかりになります</t>
         </is>
       </c>
     </row>
@@ -1141,16 +1137,16 @@
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
-      <c r="B34" s="4" t="inlineStr"/>
+      <c r="B34" s="4" t="n"/>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>使いたい色・避けたい色</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr"/>
+          <t>今の文章・写真は変更してよいですか</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="n"/>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>ブランドカラーなど。理由も一言あると助かります</t>
+          <t>誰が書いた(撮った)ものか / こちらで書き換えてよいか / 写真の使用許可は続いているか ★勝手に変えられない素材があると後で困ります</t>
         </is>
       </c>
     </row>
@@ -1158,16 +1154,16 @@
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="4" t="inlineStr"/>
-      <c r="C35" s="6" t="inlineStr">
-        <is>
-          <t>好みの書体イメージ</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr"/>
+      <c r="B35" s="4" t="n"/>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>サイトに載せたいページ・内容</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="n"/>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>例: 明朝=伝統的・上品 / ゴシック=現代的・明快 のどちら寄りか ★フォント選定に直結</t>
+          <t>思いつくものを自由に</t>
         </is>
       </c>
     </row>
@@ -1175,16 +1171,16 @@
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="4" t="inlineStr"/>
+      <c r="B36" s="4" t="n"/>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>ブランドガイドの有無</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr"/>
+          <t>必要な機能</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="n"/>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>ロゴ規定 / 指定フォント等があれば</t>
+          <t>問い合わせフォーム / 予約 / ブログ / ネット販売 など</t>
         </is>
       </c>
     </row>
@@ -1192,16 +1188,16 @@
       <c r="A37" s="2" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="4" t="inlineStr"/>
-      <c r="C37" s="6" t="inlineStr">
-        <is>
-          <t>(リニューアル)「これがあるとウチと分かる」要素</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr"/>
+      <c r="B37" s="4" t="n"/>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>必須の掲載事項</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="n"/>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>色・ロゴ・言い回しなど、残すべき“目印” ★勝手に消さないために必須</t>
+          <t>会社情報 / 資格・許認可 / 法定表記 など</t>
         </is>
       </c>
     </row>
@@ -1211,18 +1207,18 @@
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>I.体制・進行・制約</t>
-        </is>
-      </c>
-      <c r="C38" s="4" t="inlineStr">
-        <is>
-          <t>最終的に判断される方</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr"/>
+          <t>H.デザインの希望</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>サイトを見た人に「どうなってほしい」ですか</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="n"/>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>社内で公開可否を決裁される方(後の手戻り防止)</t>
+          <t>「かわいい」「かっこいい」は人によって思い浮かべるものが違います。見た方にどんな気持ち・行動になってほしいかでお聞かせください。例: 安心して問い合わせたくなる / ここなら任せられると感じる ★デザインの狙いが定まります</t>
         </is>
       </c>
     </row>
@@ -1230,16 +1226,16 @@
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="4" t="inlineStr"/>
+      <c r="B39" s="4" t="n"/>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>社内の確認フロー</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr"/>
+          <t>サイトの雰囲気・トーン</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="n"/>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>誰の確認が必要か</t>
+          <t>別シート「トーン診断」もあわせてご記入ください</t>
         </is>
       </c>
     </row>
@@ -1247,16 +1243,16 @@
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
-      <c r="B40" s="4" t="inlineStr"/>
+      <c r="B40" s="4" t="n"/>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>(リニューアル)今のサイトURL</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr"/>
+          <t>使いたい色・避けたい色</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="n"/>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>検索評価を引き継ぐため必須</t>
+          <t>ブランドカラーなど。理由も一言あると助かります</t>
         </is>
       </c>
     </row>
@@ -1264,16 +1260,16 @@
       <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
-      <c r="B41" s="4" t="inlineStr"/>
-      <c r="C41" s="4" t="inlineStr">
-        <is>
-          <t>ドメイン・サーバの現状</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr"/>
+      <c r="B41" s="4" t="n"/>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>好みの書体イメージ</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="n"/>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>今どこで管理しているか / 移すか</t>
+          <t>例: 明朝=伝統的・上品 / ゴシック=現代的・明快 のどちら寄りか ★フォント選定に直結</t>
         </is>
       </c>
     </row>
@@ -1281,16 +1277,16 @@
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
-      <c r="B42" s="4" t="inlineStr"/>
+      <c r="B42" s="4" t="n"/>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>守るべき制約・締切</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr"/>
+          <t>ブランドガイドの有無</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="n"/>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>法令 / 業界ルール / 決まっている納期など</t>
+          <t>ロゴ規定 / 指定フォント等があれば</t>
         </is>
       </c>
     </row>
@@ -1298,14 +1294,120 @@
       <c r="A43" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="B43" s="4" t="inlineStr"/>
-      <c r="C43" s="4" t="inlineStr">
+      <c r="B43" s="4" t="n"/>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>(リニューアル)「これがあるとウチと分かる」要素</t>
+        </is>
+      </c>
+      <c r="D43" s="5" t="n"/>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>色・ロゴ・言い回しなど、残すべき“目印” ★勝手に消さないために必須</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>I.体制・進行・制約</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>最終的に判断される方</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="n"/>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>社内で公開可否を決裁される方(後の手戻り防止)</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="4" t="n"/>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>社内の確認フロー</t>
+        </is>
+      </c>
+      <c r="D45" s="5" t="n"/>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>誰の確認が必要か</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="4" t="n"/>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>(リニューアル)今のサイトURL</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="n"/>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>検索評価を引き継ぐため必須</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="4" t="n"/>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>ドメイン・サーバの現状</t>
+        </is>
+      </c>
+      <c r="D47" s="5" t="n"/>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>今どこで管理しているか / 移すか</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="4" t="n"/>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>守るべき制約・締切</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="n"/>
+      <c r="E48" s="4" t="inlineStr">
+        <is>
+          <t>法令 / 業界ルール / 決まっている納期など</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="4" t="n"/>
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>その他ご要望・気になること</t>
         </is>
       </c>
-      <c r="D43" s="5" t="inlineStr"/>
-      <c r="E43" s="4" t="inlineStr">
+      <c r="D49" s="5" t="n"/>
+      <c r="E49" s="4" t="inlineStr">
         <is>
           <t>何でもご記入ください</t>
         </is>
@@ -1515,7 +1617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A15"/>
+  <dimension ref="A1:A16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -1580,27 +1682,34 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr"/>
+      <c r="A11" s="12" t="inlineStr">
+        <is>
+          <t>【素材】がついた設問は、当てはまるものを選んでご記入ください。分からない場合は空欄で構いません。</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="13" t="inlineStr">
         <is>
           <t>ご記入後の流れ</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="14" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
-        <is>
-          <t>いただいた内容をもとに、デザインの方向性（コンセプト・色・書体・参考など）を</t>
-        </is>
-      </c>
+      <c r="A14" s="14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>いただいた内容をもとに、デザインの方向性（コンセプト・色・書体・参考など）を</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>ご提案書にまとめ、すり合わせの上で制作に進みます。</t>
         </is>

</xml_diff>